<commit_message>
added new data for PRVDRS 2024-2026
</commit_message>
<xml_diff>
--- a/data/Sistema_de_Notificacion_de_Muertes_Violentas/svmvHomiEdad.xlsx
+++ b/data/Sistema_de_Notificacion_de_Muertes_Violentas/svmvHomiEdad.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gnper\Documents\ViolenciaGeneroPR\data\Sistema_de_Notificacion_de_Muertes_Violentas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1899C640-9C07-46B6-88DF-D2DA695879C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E2BB10-B3A1-4FF2-A6AB-A1D7A0A4E4E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{158DB65A-6E55-0941-A295-AA375E07226E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{158DB65A-6E55-0941-A295-AA375E07226E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -442,10 +442,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA841438-AD1F-5942-BFE3-B2D151D6E29E}">
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -473,31 +473,37 @@
       <c r="I1" s="2">
         <v>2024</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="2">
+        <v>2025</v>
+      </c>
+      <c r="K1" s="2">
+        <v>2026</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E2">
         <v>2</v>
       </c>
       <c r="F2" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G2" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H2" s="2">
         <v>3</v>
@@ -506,341 +512,407 @@
         <v>3</v>
       </c>
       <c r="J2" s="2">
+        <v>2</v>
+      </c>
+      <c r="K2" s="2">
+        <v>1</v>
+      </c>
+      <c r="L2" s="2">
         <f>SUM(B2:I2)</f>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3">
+        <v>7</v>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+      <c r="D3">
         <v>4</v>
       </c>
-      <c r="C3">
-        <v>4</v>
-      </c>
-      <c r="D3">
+      <c r="E3">
+        <v>6</v>
+      </c>
+      <c r="F3" s="2">
         <v>2</v>
-      </c>
-      <c r="E3">
-        <v>5</v>
-      </c>
-      <c r="F3" s="2">
-        <v>1</v>
       </c>
       <c r="G3" s="2">
         <v>4</v>
       </c>
       <c r="H3" s="2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I3" s="2">
         <v>2</v>
       </c>
       <c r="J3" s="2">
+        <v>2</v>
+      </c>
+      <c r="K3" s="2">
+        <v>0</v>
+      </c>
+      <c r="L3" s="2">
         <f>SUM(B3:I3)</f>
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C4">
+        <v>14</v>
+      </c>
+      <c r="D4">
+        <v>10</v>
+      </c>
+      <c r="E4">
         <v>11</v>
       </c>
-      <c r="D4">
+      <c r="F4" s="2">
+        <v>11</v>
+      </c>
+      <c r="G4" s="2">
+        <v>8</v>
+      </c>
+      <c r="H4" s="2">
         <v>3</v>
       </c>
-      <c r="E4">
-        <v>8</v>
-      </c>
-      <c r="F4" s="2">
-        <v>7</v>
-      </c>
-      <c r="G4" s="2">
-        <v>4</v>
-      </c>
-      <c r="H4" s="2">
-        <v>2</v>
-      </c>
       <c r="I4" s="2">
+        <v>6</v>
+      </c>
+      <c r="J4" s="2">
         <v>5</v>
       </c>
-      <c r="J4" s="2">
-        <f t="shared" ref="J4:J14" si="0">SUM(B4:I4)</f>
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K4" s="2">
+        <v>0</v>
+      </c>
+      <c r="L4" s="2">
+        <f t="shared" ref="L4:L14" si="0">SUM(B4:I4)</f>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C5">
         <v>5</v>
       </c>
       <c r="D5">
+        <v>10</v>
+      </c>
+      <c r="E5">
+        <v>12</v>
+      </c>
+      <c r="F5" s="2">
+        <v>10</v>
+      </c>
+      <c r="G5" s="2">
+        <v>11</v>
+      </c>
+      <c r="H5" s="2">
+        <v>9</v>
+      </c>
+      <c r="I5" s="2">
+        <v>12</v>
+      </c>
+      <c r="J5" s="2">
+        <v>8</v>
+      </c>
+      <c r="K5" s="2">
+        <v>0</v>
+      </c>
+      <c r="L5" s="2">
+        <f t="shared" si="0"/>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>11</v>
+      </c>
+      <c r="D6">
+        <v>14</v>
+      </c>
+      <c r="E6">
+        <v>8</v>
+      </c>
+      <c r="F6" s="2">
+        <v>4</v>
+      </c>
+      <c r="G6" s="2">
+        <v>14</v>
+      </c>
+      <c r="H6" s="2">
+        <v>5</v>
+      </c>
+      <c r="I6" s="2">
+        <v>9</v>
+      </c>
+      <c r="J6" s="2">
+        <v>6</v>
+      </c>
+      <c r="K6" s="2">
+        <v>1</v>
+      </c>
+      <c r="L6" s="2">
+        <f t="shared" si="0"/>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>7</v>
       </c>
-      <c r="E5">
-        <v>6</v>
-      </c>
-      <c r="F5" s="2">
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7">
+        <v>6</v>
+      </c>
+      <c r="D7">
+        <v>9</v>
+      </c>
+      <c r="E7">
+        <v>10</v>
+      </c>
+      <c r="F7" s="2">
+        <v>9</v>
+      </c>
+      <c r="G7" s="2">
+        <v>9</v>
+      </c>
+      <c r="H7" s="2">
+        <v>10</v>
+      </c>
+      <c r="I7" s="2">
+        <v>9</v>
+      </c>
+      <c r="J7" s="2">
+        <v>5</v>
+      </c>
+      <c r="K7" s="2">
+        <v>3</v>
+      </c>
+      <c r="L7" s="2">
+        <f t="shared" si="0"/>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="2">
+      <c r="B8">
+        <v>6</v>
+      </c>
+      <c r="C8">
+        <v>13</v>
+      </c>
+      <c r="D8">
+        <v>11</v>
+      </c>
+      <c r="E8">
+        <v>6</v>
+      </c>
+      <c r="F8" s="2">
+        <v>5</v>
+      </c>
+      <c r="G8" s="2">
         <v>10</v>
       </c>
-      <c r="H5" s="2">
-        <v>6</v>
-      </c>
-      <c r="I5" s="2">
+      <c r="H8" s="2">
+        <v>8</v>
+      </c>
+      <c r="I8" s="2">
+        <v>13</v>
+      </c>
+      <c r="J8" s="2">
+        <v>11</v>
+      </c>
+      <c r="K8" s="2">
+        <v>1</v>
+      </c>
+      <c r="L8" s="2">
+        <f t="shared" si="0"/>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>9</v>
       </c>
-      <c r="J5" s="2">
+      <c r="B9">
+        <v>6</v>
+      </c>
+      <c r="C9">
+        <v>8</v>
+      </c>
+      <c r="D9">
+        <v>7</v>
+      </c>
+      <c r="E9">
+        <v>6</v>
+      </c>
+      <c r="F9" s="2">
+        <v>5</v>
+      </c>
+      <c r="G9" s="2">
+        <v>6</v>
+      </c>
+      <c r="H9" s="2">
+        <v>7</v>
+      </c>
+      <c r="I9" s="2">
+        <v>10</v>
+      </c>
+      <c r="J9" s="2">
+        <v>6</v>
+      </c>
+      <c r="K9" s="2">
+        <v>0</v>
+      </c>
+      <c r="L9" s="2">
         <f t="shared" si="0"/>
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>3</v>
-      </c>
-      <c r="C6">
-        <v>7</v>
-      </c>
-      <c r="D6">
-        <v>9</v>
-      </c>
-      <c r="E6">
-        <v>6</v>
-      </c>
-      <c r="F6" s="2">
-        <v>2</v>
-      </c>
-      <c r="G6" s="2">
-        <v>12</v>
-      </c>
-      <c r="H6" s="2">
-        <v>3</v>
-      </c>
-      <c r="I6" s="2">
-        <v>8</v>
-      </c>
-      <c r="J6" s="2">
-        <f t="shared" si="0"/>
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7">
-        <v>6</v>
-      </c>
-      <c r="D7">
-        <v>5</v>
-      </c>
-      <c r="E7">
-        <v>5</v>
-      </c>
-      <c r="F7" s="2">
-        <v>4</v>
-      </c>
-      <c r="G7" s="2">
-        <v>5</v>
-      </c>
-      <c r="H7" s="2">
-        <v>6</v>
-      </c>
-      <c r="I7" s="2">
-        <v>8</v>
-      </c>
-      <c r="J7" s="2">
-        <f t="shared" si="0"/>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
-        <v>2</v>
-      </c>
-      <c r="C8">
-        <v>9</v>
-      </c>
-      <c r="D8">
-        <v>6</v>
-      </c>
-      <c r="E8">
-        <v>5</v>
-      </c>
-      <c r="F8" s="2">
-        <v>4</v>
-      </c>
-      <c r="G8" s="2">
-        <v>3</v>
-      </c>
-      <c r="H8" s="2">
-        <v>5</v>
-      </c>
-      <c r="I8" s="2">
-        <v>4</v>
-      </c>
-      <c r="J8" s="2">
-        <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>1</v>
-      </c>
-      <c r="C9">
-        <v>4</v>
-      </c>
-      <c r="D9">
-        <v>3</v>
-      </c>
-      <c r="E9">
-        <v>5</v>
-      </c>
-      <c r="F9" s="2">
-        <v>2</v>
-      </c>
-      <c r="G9" s="2">
-        <v>5</v>
-      </c>
-      <c r="H9" s="2">
-        <v>5</v>
-      </c>
-      <c r="I9" s="2">
-        <v>5</v>
-      </c>
-      <c r="J9" s="2">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>10</v>
       </c>
       <c r="B10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C10">
+        <v>10</v>
+      </c>
+      <c r="D10">
+        <v>11</v>
+      </c>
+      <c r="E10">
         <v>3</v>
       </c>
-      <c r="D10">
-        <v>2</v>
-      </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
       <c r="F10" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G10" s="2">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H10" s="2">
+        <v>13</v>
+      </c>
+      <c r="I10" s="2">
+        <v>11</v>
+      </c>
+      <c r="J10" s="2">
+        <v>9</v>
+      </c>
+      <c r="K10" s="2">
         <v>3</v>
       </c>
-      <c r="I10" s="2">
-        <v>5</v>
-      </c>
-      <c r="J10" s="2">
+      <c r="L10" s="2">
         <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>11</v>
       </c>
       <c r="B11">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C11">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E11">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F11" s="2">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G11" s="2">
+        <v>6</v>
+      </c>
+      <c r="H11" s="2">
+        <v>6</v>
+      </c>
+      <c r="I11" s="2">
         <v>3</v>
       </c>
-      <c r="H11" s="2">
-        <v>1</v>
-      </c>
-      <c r="I11" s="2">
-        <v>1</v>
-      </c>
       <c r="J11" s="2">
+        <v>13</v>
+      </c>
+      <c r="K11" s="2">
+        <v>0</v>
+      </c>
+      <c r="L11" s="2">
         <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>12</v>
       </c>
       <c r="B12">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="C12">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="E12">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="F12" s="2">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G12" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H12" s="2">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="I12" s="2">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="J12" s="2">
+        <v>24</v>
+      </c>
+      <c r="K12" s="2">
+        <v>6</v>
+      </c>
+      <c r="L12" s="2">
         <f t="shared" si="0"/>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -851,13 +923,13 @@
         <v>0</v>
       </c>
       <c r="D13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13">
         <v>0</v>
       </c>
       <c r="F13" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" s="2">
         <v>0</v>
@@ -869,49 +941,63 @@
         <v>0</v>
       </c>
       <c r="J13" s="2">
+        <v>0</v>
+      </c>
+      <c r="K13" s="2">
+        <v>0</v>
+      </c>
+      <c r="L13" s="2">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>14</v>
       </c>
       <c r="B14">
         <f>SUM(B2:B13)</f>
-        <v>36</v>
+        <v>90</v>
       </c>
       <c r="C14">
         <f>SUM(C2:C13)</f>
-        <v>53</v>
+        <v>97</v>
       </c>
       <c r="D14">
         <f>SUM(D2:D13)</f>
-        <v>41</v>
+        <v>97</v>
       </c>
       <c r="E14">
         <f>SUM(E2:E13)</f>
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="F14" s="2">
         <f t="shared" ref="F14" si="1">SUM(F2:F13)</f>
-        <v>37</v>
+        <v>69</v>
       </c>
       <c r="G14" s="2">
         <f>SUM(G2:G13)</f>
-        <v>53</v>
+        <v>84</v>
       </c>
       <c r="H14" s="2">
         <f>SUM(H2:H13)</f>
-        <v>47</v>
+        <v>92</v>
       </c>
       <c r="I14" s="2">
         <f>SUM(I2:I13)</f>
-        <v>58</v>
+        <v>100</v>
       </c>
       <c r="J14" s="2">
-        <f t="shared" si="0"/>
-        <v>374</v>
+        <f t="shared" ref="J14:K14" si="2">SUM(J2:J13)</f>
+        <v>91</v>
+      </c>
+      <c r="K14" s="2">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+      <c r="L14" s="2">
+        <f>SUM(B14:K14)</f>
+        <v>821</v>
       </c>
     </row>
   </sheetData>

</xml_diff>